<commit_message>
fix(N-03): surface PowerPoint discovery, routing, and pptx proof
Make PowerPoint discoverable in home/お願い presets and format pickers,
route natural JP PowerPoint intents to required pptx export, add openable
LP .pptx proof sample, and add N-03 Production probe + CI Quality Gate.

Co-authored-by: shenmixingye08-design <shenmixingye08-design@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/samples/cost-table.xlsx
+++ b/public/samples/cost-table.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="データ" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="ピボット集計" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
   <si>
     <t>項目</t>
   </si>
@@ -31,9 +32,6 @@
     <t>マーケ</t>
   </si>
   <si>
-    <t>48000</t>
-  </si>
-  <si>
     <t>見本値</t>
   </si>
   <si>
@@ -43,41 +41,35 @@
     <t>制作</t>
   </si>
   <si>
-    <t>120000</t>
-  </si>
-  <si>
     <t>通信費</t>
   </si>
   <si>
     <t>固定</t>
   </si>
   <si>
-    <t>12800</t>
-  </si>
-  <si>
     <t>交通費</t>
   </si>
   <si>
     <t>変動</t>
   </si>
   <si>
-    <t>8600</t>
-  </si>
-  <si>
     <t>雑費</t>
   </si>
   <si>
     <t>その他</t>
   </si>
   <si>
-    <t>5400</t>
+    <t>合計</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;¥&quot;#,##0"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -92,6 +84,11 @@
       <name val="Yu Gothic"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Yu Gothic"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Yu Gothic"/>
     </font>
@@ -136,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -148,6 +145,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -163,6 +164,115 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="ja-JP"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ja-JP" sz="1200"/>
+              <a:t>カテゴリ別合計</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ピボット集計'!$B$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ピボット集計'!$A$2:$A$6</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ピボット集計'!$B$2:$B$6</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="ATLAS Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -516,67 +626,67 @@
       <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5">
+        <v>48000</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
+      <c r="C3" s="5">
+        <v>120000</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="5">
+        <v>12800</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="C5" s="5">
+        <v>8600</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
+      </c>
+      <c r="C6" s="5">
+        <v>5400</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -584,4 +694,68 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>8600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>12800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rIdAtlasChart"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(N-03): surface PowerPoint discovery, routing, and pptx proof (#255)
* fix(N-03): surface PowerPoint discovery, routing, and pptx proof

Make PowerPoint discoverable in home/お願い presets and format pickers,
route natural JP PowerPoint intents to required pptx export, add openable
LP .pptx proof sample, and add N-03 Production probe + CI Quality Gate.

Co-authored-by: shenmixingye08-design <shenmixingye08-design@users.noreply.github.com>

* test(N-03): align expectations with PowerPoint surface

Update proof catalog and quick-preset assertions for pptx exposure,
and refresh measured landing sample artifacts from the generator path.

Co-authored-by: shenmixingye08-design <shenmixingye08-design@users.noreply.github.com>

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: shenmixingye08-design <shenmixingye08-design@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/samples/cost-table.xlsx
+++ b/public/samples/cost-table.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="データ" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="ピボット集計" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
   <si>
     <t>項目</t>
   </si>
@@ -31,9 +32,6 @@
     <t>マーケ</t>
   </si>
   <si>
-    <t>48000</t>
-  </si>
-  <si>
     <t>見本値</t>
   </si>
   <si>
@@ -43,41 +41,35 @@
     <t>制作</t>
   </si>
   <si>
-    <t>120000</t>
-  </si>
-  <si>
     <t>通信費</t>
   </si>
   <si>
     <t>固定</t>
   </si>
   <si>
-    <t>12800</t>
-  </si>
-  <si>
     <t>交通費</t>
   </si>
   <si>
     <t>変動</t>
   </si>
   <si>
-    <t>8600</t>
-  </si>
-  <si>
     <t>雑費</t>
   </si>
   <si>
     <t>その他</t>
   </si>
   <si>
-    <t>5400</t>
+    <t>合計</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;¥&quot;#,##0"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -92,6 +84,11 @@
       <name val="Yu Gothic"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Yu Gothic"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Yu Gothic"/>
     </font>
@@ -136,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -148,6 +145,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -163,6 +164,115 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="ja-JP"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ja-JP" sz="1200"/>
+              <a:t>カテゴリ別合計</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ピボット集計'!$B$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ピボット集計'!$A$2:$A$6</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ピボット集計'!$B$2:$B$6</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="ATLAS Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -516,67 +626,67 @@
       <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5">
+        <v>48000</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
+      <c r="C3" s="5">
+        <v>120000</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="5">
+        <v>12800</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="C5" s="5">
+        <v>8600</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
+      </c>
+      <c r="C6" s="5">
+        <v>5400</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -584,4 +694,68 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>8600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>12800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rIdAtlasChart"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: close typecheck, lint, and redaction regression gaps
Make tick schema apply use the existing migration helper shape, keep
DispatchResult.deferred compatible with existing mocks, and accept
[redacted-token] in structured-log assertions.

Co-authored-by: shenmixingye08-design <shenmixingye08-design@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/samples/cost-table.xlsx
+++ b/public/samples/cost-table.xlsx
@@ -5,14 +5,16 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="データ" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="ピボット集計" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'データ'!$1:$1</definedName>
+  </definedNames>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>項目</t>
   </si>
@@ -57,9 +59,6 @@
   </si>
   <si>
     <t>その他</t>
-  </si>
-  <si>
-    <t>合計</t>
   </si>
 </sst>
 </file>
@@ -69,7 +68,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;¥&quot;#,##0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -84,11 +83,6 @@
       <name val="Yu Gothic"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Yu Gothic"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Yu Gothic"/>
     </font>
@@ -133,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -148,7 +142,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -164,115 +157,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:lang val="ja-JP"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1200"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="ja-JP" sz="1200"/>
-              <a:t>カテゴリ別合計</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'ピボット集計'!$B$1</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:cat>
-            <c:strRef>
-              <c:f>'ピボット集計'!$A$2:$A$6</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'ピボット集計'!$B$2:$B$6</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:axId val="1"/>
-        <c:axId val="2"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:crossAx val="2"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="2"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:crossAx val="1"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-  </c:chart>
-</c:chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame>
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="ATLAS Chart 1"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -597,6 +481,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -605,7 +492,7 @@
     <col min="4" max="4" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -619,7 +506,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="18" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -633,7 +520,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="18" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
@@ -647,7 +534,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="18" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -661,7 +548,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="18" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -675,7 +562,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="18" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -691,71 +578,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D6"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
-        <v>120000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3">
-        <v>8600</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>48000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
-        <v>5400</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>12800</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rIdAtlasChart"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>